<commit_message>
Change column names, etc.
</commit_message>
<xml_diff>
--- a/data-raw/BeatlesSchema.xlsx
+++ b/data-raw/BeatlesSchema.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/PFUPipelineTools/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA5D3C8-6030-B94E-BB8B-ABB9DA7C757B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66553C40-4671-0947-8C17-C42A187B27C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22060" yWindow="500" windowWidth="18920" windowHeight="16440" activeTab="1" xr2:uid="{8A3A5368-3B53-8E41-9868-764DDCC0B41C}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
-    <sheet name="Schema" sheetId="1" r:id="rId2"/>
+    <sheet name="SchemaTable" sheetId="1" r:id="rId2"/>
     <sheet name="Member" sheetId="2" r:id="rId3"/>
     <sheet name="Role" sheetId="3" r:id="rId4"/>
   </sheets>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="25">
   <si>
-    <t>Table</t>
-  </si>
-  <si>
     <t>int</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t>ColDataType</t>
+  </si>
+  <si>
+    <t>TableName</t>
   </si>
 </sst>
 </file>
@@ -501,17 +501,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -531,142 +531,142 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="b">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
         <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" t="b">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -682,10 +682,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -693,7 +693,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -701,7 +701,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -709,7 +709,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -717,7 +717,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -733,10 +733,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -744,7 +744,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -752,7 +752,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -760,7 +760,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -768,7 +768,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>